<commit_message>
Fix CAPEX/OPEX workbooks showing no totals in non-recalculating viewers
Two issues combined to make the totals invisible: (1) the workbook opened
on the text-only Instructions/使用说明 tab by default instead of Summary/
总览, and (2) openpyxl writes an empty <v/> placeholder for every formula
cell with no cached result, which viewers that don't run their own
recalculation (mobile quick-look style previews) render as blank rather
than a number.

Fixed by defaulting the active sheet to Summary/总览, and adding
bake_cache.py, which uses the `formulas` library to compute every formula
and writes the real cached value into the cell XML after generation --
Excel/Sheets/LibreOffice still recalculate live since the formulas are
untouched, but now a non-recalculating viewer shows the correct numbers
immediately.
</commit_message>
<xml_diff>
--- a/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
+++ b/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="C6" s="4">
         <f>'CAPEX 开店资本支出'!E68</f>
-        <v/>
+        <v>89462.5</v>
       </c>
     </row>
     <row r="8">
@@ -615,7 +615,7 @@
       </c>
       <c r="C9" s="4">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
     </row>
     <row r="10">
@@ -626,7 +626,7 @@
       </c>
       <c r="C10" s="5">
         <f>'OPEX 每月营运支出'!C56</f>
-        <v/>
+        <v>23212.5</v>
       </c>
     </row>
     <row r="12">
@@ -644,7 +644,7 @@
       </c>
       <c r="C13" s="4">
         <f>'CAPEX 开店资本支出'!E68</f>
-        <v/>
+        <v>89462.5</v>
       </c>
     </row>
     <row r="14">
@@ -653,9 +653,9 @@
           <t>对比 RM50,000-100,000 预算区间</t>
         </is>
       </c>
-      <c r="C14">
+      <c r="C14" t="str">
         <f>IF(C13&lt;='关键假设'!C4,"低于下限，资金充裕",IF(C13&lt;='关键假设'!C5,"落在预算区间内","超出预算上限，需调整假设或增资"))</f>
-        <v/>
+        <v>落在预算区间内</v>
       </c>
     </row>
     <row r="17">
@@ -673,7 +673,7 @@
       </c>
       <c r="C18" s="5">
         <f>'12个月现金流预测'!N10</f>
-        <v/>
+        <v>890549.8549865913</v>
       </c>
     </row>
     <row r="19">
@@ -684,7 +684,7 @@
       </c>
       <c r="C19" s="5">
         <f>'12个月现金流预测'!N15</f>
-        <v/>
+        <v>19949.40863823614</v>
       </c>
     </row>
     <row r="20">
@@ -695,7 +695,7 @@
       </c>
       <c r="C20" s="5">
         <f>'12个月现金流预测'!M16</f>
-        <v/>
+        <v>19949.40863823614</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="E5" s="14">
         <f>C5*D5</f>
-        <v/>
+        <v>6000.0</v>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="E6" s="14">
         <f>C6*D6</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="F6" s="7" t="inlineStr"/>
     </row>
@@ -1384,7 +1384,7 @@
       </c>
       <c r="E7" s="14">
         <f>C7*D7</f>
-        <v/>
+        <v>1000.0</v>
       </c>
       <c r="F7" s="7" t="inlineStr"/>
     </row>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="E8" s="14">
         <f>C8*D8</f>
-        <v/>
+        <v>800.0</v>
       </c>
       <c r="F8" s="7" t="inlineStr"/>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="E9" s="14">
         <f>C9*D9</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="F9" s="7" t="inlineStr"/>
     </row>
@@ -1434,7 +1434,7 @@
       <c r="D10" s="16" t="n"/>
       <c r="E10" s="17">
         <f>SUM(E5:E9)</f>
-        <v/>
+        <v>8800.0</v>
       </c>
     </row>
     <row r="12">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="E14" s="14">
         <f>C14*D14</f>
-        <v/>
+        <v>2400.0</v>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="E15" s="14">
         <f>C15*D15</f>
-        <v/>
+        <v>1200.0</v>
       </c>
       <c r="F15" s="7" t="inlineStr"/>
     </row>
@@ -1525,7 +1525,7 @@
       </c>
       <c r="E16" s="14">
         <f>C16*D16</f>
-        <v/>
+        <v>2500.0</v>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
     </row>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="E17" s="14">
         <f>C17*D17</f>
-        <v/>
+        <v>1000.0</v>
       </c>
       <c r="F17" s="7" t="inlineStr"/>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="E18" s="14">
         <f>C18*D18</f>
-        <v/>
+        <v>800.0</v>
       </c>
       <c r="F18" s="7" t="inlineStr"/>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="E19" s="14">
         <f>C19*D19</f>
-        <v/>
+        <v>1500.0</v>
       </c>
       <c r="F19" s="7" t="inlineStr"/>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="E20" s="14">
         <f>C20*D20</f>
-        <v/>
+        <v>1000.0</v>
       </c>
       <c r="F20" s="7" t="inlineStr"/>
     </row>
@@ -1611,7 +1611,7 @@
       <c r="D21" s="16" t="n"/>
       <c r="E21" s="17">
         <f>SUM(E14:E20)</f>
-        <v/>
+        <v>10400.0</v>
       </c>
     </row>
     <row r="23">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="E25" s="14">
         <f>C25*D25</f>
-        <v/>
+        <v>900.0</v>
       </c>
       <c r="F25" s="7" t="inlineStr"/>
     </row>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="E26" s="14">
         <f>C26*D26</f>
-        <v/>
+        <v>2200.0</v>
       </c>
       <c r="F26" s="7" t="inlineStr"/>
     </row>
@@ -1698,7 +1698,7 @@
       </c>
       <c r="E27" s="14">
         <f>C27*D27</f>
-        <v/>
+        <v>400.0</v>
       </c>
       <c r="F27" s="7" t="inlineStr"/>
     </row>
@@ -1716,7 +1716,7 @@
       </c>
       <c r="E28" s="14">
         <f>C28*D28</f>
-        <v/>
+        <v>250.0</v>
       </c>
       <c r="F28" s="7" t="inlineStr"/>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="E29" s="14">
         <f>C29*D29</f>
-        <v/>
+        <v>200.0</v>
       </c>
       <c r="F29" s="7" t="inlineStr"/>
     </row>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="E30" s="14">
         <f>C30*D30</f>
-        <v/>
+        <v>600.0</v>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
       </c>
       <c r="E31" s="14">
         <f>C31*D31</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="F31" s="7" t="inlineStr"/>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="E32" s="14">
         <f>C32*D32</f>
-        <v/>
+        <v>300.0</v>
       </c>
       <c r="F32" s="7" t="inlineStr"/>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E33" s="14">
         <f>C33*D33</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="F33" s="7" t="inlineStr"/>
     </row>
@@ -1824,7 +1824,7 @@
       <c r="D34" s="16" t="n"/>
       <c r="E34" s="17">
         <f>SUM(E25:E33)</f>
-        <v/>
+        <v>5850.0</v>
       </c>
     </row>
     <row r="36">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="E38" s="14">
         <f>C38*D38</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
       </c>
       <c r="E39" s="14">
         <f>C39*D39</f>
-        <v/>
+        <v>300.0</v>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="E40" s="14">
         <f>C40*D40</f>
-        <v/>
+        <v>300.0</v>
       </c>
       <c r="F40" s="7" t="inlineStr"/>
     </row>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="E41" s="14">
         <f>C41*D41</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="F41" s="7" t="inlineStr"/>
     </row>
@@ -1955,7 +1955,7 @@
       </c>
       <c r="E42" s="14">
         <f>C42*D42</f>
-        <v/>
+        <v>3000.0</v>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
@@ -1973,7 +1973,7 @@
       <c r="D43" s="16" t="n"/>
       <c r="E43" s="17">
         <f>SUM(E38:E42)</f>
-        <v/>
+        <v>3600.0</v>
       </c>
     </row>
     <row r="45">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="E47" s="14">
         <f>C47*D47</f>
-        <v/>
+        <v>300.0</v>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="E48" s="14">
         <f>C48*D48</f>
-        <v/>
+        <v>500.0</v>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="E49" s="14">
         <f>C49*D49</f>
-        <v/>
+        <v>300.0</v>
       </c>
       <c r="F49" s="7" t="inlineStr"/>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="E50" s="14">
         <f>C50*D50</f>
-        <v/>
+        <v>1500.0</v>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="E51" s="14">
         <f>C51*D51</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
@@ -2126,7 +2126,7 @@
       <c r="D52" s="16" t="n"/>
       <c r="E52" s="17">
         <f>SUM(E47:E51)</f>
-        <v/>
+        <v>2600.0</v>
       </c>
     </row>
     <row r="54">
@@ -2173,7 +2173,7 @@
       <c r="D56" s="9" t="n"/>
       <c r="E56" s="14">
         <f>'关键假设'!C21*'关键假设'!C18</f>
-        <v/>
+        <v>24500.0</v>
       </c>
       <c r="F56" s="7" t="inlineStr">
         <is>
@@ -2191,7 +2191,7 @@
       <c r="D57" s="9" t="n"/>
       <c r="E57" s="14">
         <f>'关键假设'!C21*'关键假设'!C19</f>
-        <v/>
+        <v>7000.0</v>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
       <c r="D58" s="9" t="n"/>
       <c r="E58" s="14">
         <f>'关键假设'!C21*'关键假设'!C20</f>
-        <v/>
+        <v>3500.0</v>
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
@@ -2227,7 +2227,7 @@
       <c r="D59" s="16" t="n"/>
       <c r="E59" s="17">
         <f>SUM(E56:E58)</f>
-        <v/>
+        <v>35000.0</v>
       </c>
     </row>
     <row r="61">
@@ -2278,7 +2278,7 @@
       </c>
       <c r="E63" s="14">
         <f>C63*D63</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="F63" s="7" t="inlineStr">
         <is>
@@ -2296,7 +2296,7 @@
       <c r="D64" s="16" t="n"/>
       <c r="E64" s="17">
         <f>'OPEX 每月营运支出'!C56</f>
-        <v/>
+        <v>23212.5</v>
       </c>
     </row>
     <row r="67">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="E68" s="19">
         <f>E10+E21+E34+E43+E52+E59+E64</f>
-        <v/>
+        <v>89462.5</v>
       </c>
     </row>
     <row r="69">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="E69" s="21">
         <f>'关键假设'!C4-E68</f>
-        <v/>
+        <v>-39462.5</v>
       </c>
     </row>
     <row r="70">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E70" s="21">
         <f>'关键假设'!C5-E68</f>
-        <v/>
+        <v>10537.5</v>
       </c>
     </row>
   </sheetData>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="C11" s="17">
         <f>SUM(C5:C10)</f>
-        <v/>
+        <v>4850.0</v>
       </c>
     </row>
     <row r="13">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="C15" s="14">
         <f>'关键假设'!C41</f>
-        <v/>
+        <v>2000.0</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
@@ -2530,7 +2530,7 @@
       </c>
       <c r="C16" s="14">
         <f>'关键假设'!C41*'关键假设'!C42</f>
-        <v/>
+        <v>260.0</v>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C18" s="17">
         <f>SUM(C15:C17)</f>
-        <v/>
+        <v>2560.0</v>
       </c>
     </row>
     <row r="20">
@@ -2611,7 +2611,7 @@
       </c>
       <c r="C23" s="17">
         <f>SUM(C22:C22)</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="25">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="C30" s="17">
         <f>SUM(C27:C29)</f>
-        <v/>
+        <v>1000.0</v>
       </c>
     </row>
     <row r="32">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="C37" s="17">
         <f>SUM(C34:C36)</f>
-        <v/>
+        <v>125.0</v>
       </c>
     </row>
     <row r="39">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="C44" s="17">
         <f>SUM(C41:C43)</f>
-        <v/>
+        <v>450.0</v>
       </c>
     </row>
     <row r="46">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="C51" s="17">
         <f>SUM(C48:C50)</f>
-        <v/>
+        <v>300.0</v>
       </c>
     </row>
     <row r="54">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="C55" s="19">
         <f>C11+C18+C23+C30+C37+C44+C51</f>
-        <v/>
+        <v>9285.0</v>
       </c>
     </row>
     <row r="56">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="C56" s="21">
         <f>C55*2.5</f>
-        <v/>
+        <v>23212.5</v>
       </c>
     </row>
   </sheetData>
@@ -3059,55 +3059,55 @@
       </c>
       <c r="B4" s="23">
         <f>'关键假设'!C24</f>
-        <v/>
+        <v>40.0</v>
       </c>
       <c r="C4" s="23">
         <f>B4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>41.2</v>
       </c>
       <c r="D4" s="23">
         <f>C4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>42.43600000000001</v>
       </c>
       <c r="E4" s="23">
         <f>D4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>43.70908000000001</v>
       </c>
       <c r="F4" s="23">
         <f>E4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>45.02035240000001</v>
       </c>
       <c r="G4" s="23">
         <f>F4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>46.37096297200001</v>
       </c>
       <c r="H4" s="23">
         <f>G4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>47.76209186116001</v>
       </c>
       <c r="I4" s="23">
         <f>H4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>49.19495461699481</v>
       </c>
       <c r="J4" s="23">
         <f>I4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>50.67080325550466</v>
       </c>
       <c r="K4" s="23">
         <f>J4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>52.1909273531698</v>
       </c>
       <c r="L4" s="23">
         <f>K4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>53.75665517376489</v>
       </c>
       <c r="M4" s="23">
         <f>L4*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>55.36935482897784</v>
       </c>
       <c r="N4" s="24">
         <f>SUM(B4:M4)</f>
-        <v/>
+        <v>567.681182461572</v>
       </c>
     </row>
     <row r="5">
@@ -3118,51 +3118,51 @@
       </c>
       <c r="B5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="C5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="D5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="E5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="F5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="G5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="H5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="I5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="J5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="K5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="L5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
       <c r="M5" s="5">
         <f>'关键假设'!C25</f>
-        <v/>
+        <v>1400.0</v>
       </c>
     </row>
     <row r="6">
@@ -3173,55 +3173,55 @@
       </c>
       <c r="B6" s="5">
         <f>B4*B5</f>
-        <v/>
+        <v>56000.0</v>
       </c>
       <c r="C6" s="5">
         <f>C4*C5</f>
-        <v/>
+        <v>57680.00000000001</v>
       </c>
       <c r="D6" s="5">
         <f>D4*D5</f>
-        <v/>
+        <v>59410.40000000001</v>
       </c>
       <c r="E6" s="5">
         <f>E4*E5</f>
-        <v/>
+        <v>61192.71200000001</v>
       </c>
       <c r="F6" s="5">
         <f>F4*F5</f>
-        <v/>
+        <v>63028.49336000001</v>
       </c>
       <c r="G6" s="5">
         <f>G4*G5</f>
-        <v/>
+        <v>64919.348160800015</v>
       </c>
       <c r="H6" s="5">
         <f>H4*H5</f>
-        <v/>
+        <v>66866.92860562401</v>
       </c>
       <c r="I6" s="5">
         <f>I4*I5</f>
-        <v/>
+        <v>68872.93646379274</v>
       </c>
       <c r="J6" s="5">
         <f>J4*J5</f>
-        <v/>
+        <v>70939.12455770653</v>
       </c>
       <c r="K6" s="5">
         <f>K4*K5</f>
-        <v/>
+        <v>73067.29829443771</v>
       </c>
       <c r="L6" s="5">
         <f>L4*L5</f>
-        <v/>
+        <v>75259.31724327085</v>
       </c>
       <c r="M6" s="5">
         <f>M4*M5</f>
-        <v/>
+        <v>77517.09676056898</v>
       </c>
       <c r="N6" s="25">
         <f>SUM(B6:M6)</f>
-        <v/>
+        <v>794753.6554462009</v>
       </c>
     </row>
     <row r="7">
@@ -3232,55 +3232,55 @@
       </c>
       <c r="B7" s="23">
         <f>'关键假设'!C26</f>
-        <v/>
+        <v>150.0</v>
       </c>
       <c r="C7" s="23">
         <f>B7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>154.5</v>
       </c>
       <c r="D7" s="23">
         <f>C7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>159.135</v>
       </c>
       <c r="E7" s="23">
         <f>D7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>163.90905</v>
       </c>
       <c r="F7" s="23">
         <f>E7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>168.8263215</v>
       </c>
       <c r="G7" s="23">
         <f>F7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>173.891111145</v>
       </c>
       <c r="H7" s="23">
         <f>G7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>179.10784447935</v>
       </c>
       <c r="I7" s="23">
         <f>H7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>184.4810798137305</v>
       </c>
       <c r="J7" s="23">
         <f>I7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>190.0155122081424</v>
       </c>
       <c r="K7" s="23">
         <f>J7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>195.7159775743867</v>
       </c>
       <c r="L7" s="23">
         <f>K7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>201.5874569016183</v>
       </c>
       <c r="M7" s="23">
         <f>L7*(1+'关键假设'!C28)</f>
-        <v/>
+        <v>207.63508060866687</v>
       </c>
       <c r="N7" s="24">
         <f>SUM(B7:M7)</f>
-        <v/>
+        <v>2128.804434230895</v>
       </c>
     </row>
     <row r="8">
@@ -3291,51 +3291,51 @@
       </c>
       <c r="B8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="C8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="D8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="E8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="F8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="G8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="H8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="I8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="J8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="K8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="L8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="M8" s="5">
         <f>'关键假设'!C27</f>
-        <v/>
+        <v>45.0</v>
       </c>
     </row>
     <row r="9">
@@ -3346,55 +3346,55 @@
       </c>
       <c r="B9" s="5">
         <f>B7*B8</f>
-        <v/>
+        <v>6750.0</v>
       </c>
       <c r="C9" s="5">
         <f>C7*C8</f>
-        <v/>
+        <v>6952.5</v>
       </c>
       <c r="D9" s="5">
         <f>D7*D8</f>
-        <v/>
+        <v>7161.075</v>
       </c>
       <c r="E9" s="5">
         <f>E7*E8</f>
-        <v/>
+        <v>7375.90725</v>
       </c>
       <c r="F9" s="5">
         <f>F7*F8</f>
-        <v/>
+        <v>7597.1844675</v>
       </c>
       <c r="G9" s="5">
         <f>G7*G8</f>
-        <v/>
+        <v>7825.100001525</v>
       </c>
       <c r="H9" s="5">
         <f>H7*H8</f>
-        <v/>
+        <v>8059.85300157075</v>
       </c>
       <c r="I9" s="5">
         <f>I7*I8</f>
-        <v/>
+        <v>8301.648591617872</v>
       </c>
       <c r="J9" s="5">
         <f>J7*J8</f>
-        <v/>
+        <v>8550.698049366409</v>
       </c>
       <c r="K9" s="5">
         <f>K7*K8</f>
-        <v/>
+        <v>8807.218990847401</v>
       </c>
       <c r="L9" s="5">
         <f>L7*L8</f>
-        <v/>
+        <v>9071.435560572823</v>
       </c>
       <c r="M9" s="5">
         <f>M7*M8</f>
-        <v/>
+        <v>9343.578627390008</v>
       </c>
       <c r="N9" s="25">
         <f>SUM(B9:M9)</f>
-        <v/>
+        <v>95796.19954039025</v>
       </c>
     </row>
     <row r="10">
@@ -3405,55 +3405,55 @@
       </c>
       <c r="B10" s="17">
         <f>B6+B9</f>
-        <v/>
+        <v>62750.0</v>
       </c>
       <c r="C10" s="17">
         <f>C6+C9</f>
-        <v/>
+        <v>64632.50000000001</v>
       </c>
       <c r="D10" s="17">
         <f>D6+D9</f>
-        <v/>
+        <v>66571.475</v>
       </c>
       <c r="E10" s="17">
         <f>E6+E9</f>
-        <v/>
+        <v>68568.61925</v>
       </c>
       <c r="F10" s="17">
         <f>F6+F9</f>
-        <v/>
+        <v>70625.67782750001</v>
       </c>
       <c r="G10" s="17">
         <f>G6+G9</f>
-        <v/>
+        <v>72744.44816232502</v>
       </c>
       <c r="H10" s="17">
         <f>H6+H9</f>
-        <v/>
+        <v>74926.78160719476</v>
       </c>
       <c r="I10" s="17">
         <f>I6+I9</f>
-        <v/>
+        <v>77174.5850554106</v>
       </c>
       <c r="J10" s="17">
         <f>J6+J9</f>
-        <v/>
+        <v>79489.82260707294</v>
       </c>
       <c r="K10" s="17">
         <f>K6+K9</f>
-        <v/>
+        <v>81874.51728528511</v>
       </c>
       <c r="L10" s="17">
         <f>L6+L9</f>
-        <v/>
+        <v>84330.75280384367</v>
       </c>
       <c r="M10" s="17">
         <f>M6+M9</f>
-        <v/>
+        <v>86860.675387959</v>
       </c>
       <c r="N10" s="25">
         <f>SUM(B10:M10)</f>
-        <v/>
+        <v>890549.8549865913</v>
       </c>
     </row>
     <row r="11">
@@ -3464,55 +3464,55 @@
       </c>
       <c r="B11" s="5">
         <f>(B6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(B9*'关键假设'!C15)</f>
-        <v/>
+        <v>10400.0</v>
       </c>
       <c r="C11" s="5">
         <f>(C6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(C9*'关键假设'!C15)</f>
-        <v/>
+        <v>10712.000000000002</v>
       </c>
       <c r="D11" s="5">
         <f>(D6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(D9*'关键假设'!C15)</f>
-        <v/>
+        <v>11033.360000000002</v>
       </c>
       <c r="E11" s="5">
         <f>(E6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(E9*'关键假设'!C15)</f>
-        <v/>
+        <v>11364.360800000002</v>
       </c>
       <c r="F11" s="5">
         <f>(F6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(F9*'关键假设'!C15)</f>
-        <v/>
+        <v>11705.291624000001</v>
       </c>
       <c r="G11" s="5">
         <f>(G6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(G9*'关键假设'!C15)</f>
-        <v/>
+        <v>12056.450372720003</v>
       </c>
       <c r="H11" s="5">
         <f>(H6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(H9*'关键假设'!C15)</f>
-        <v/>
+        <v>12418.143883901603</v>
       </c>
       <c r="I11" s="5">
         <f>(I6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(I9*'关键假设'!C15)</f>
-        <v/>
+        <v>12790.688200418652</v>
       </c>
       <c r="J11" s="5">
         <f>(J6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(J9*'关键假设'!C15)</f>
-        <v/>
+        <v>13174.408846431212</v>
       </c>
       <c r="K11" s="5">
         <f>(K6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(K9*'关键假设'!C15)</f>
-        <v/>
+        <v>13569.641111824147</v>
       </c>
       <c r="L11" s="5">
         <f>(L6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(L9*'关键假设'!C15)</f>
-        <v/>
+        <v>13976.730345178872</v>
       </c>
       <c r="M11" s="5">
         <f>(M6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(M9*'关键假设'!C15)</f>
-        <v/>
+        <v>14396.032255534239</v>
       </c>
       <c r="N11" s="25">
         <f>SUM(B11:M11)</f>
-        <v/>
+        <v>147597.10744000872</v>
       </c>
     </row>
     <row r="12">
@@ -3523,55 +3523,55 @@
       </c>
       <c r="B12" s="5">
         <f>B10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>831.4375</v>
       </c>
       <c r="C12" s="5">
         <f>C10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>856.3806250000001</v>
       </c>
       <c r="D12" s="5">
         <f>D10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>882.07204375</v>
       </c>
       <c r="E12" s="5">
         <f>E10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>908.5342050625001</v>
       </c>
       <c r="F12" s="5">
         <f>F10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>935.7902312143751</v>
       </c>
       <c r="G12" s="5">
         <f>G10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>963.8639381508065</v>
       </c>
       <c r="H12" s="5">
         <f>H10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>992.7798562953305</v>
       </c>
       <c r="I12" s="5">
         <f>I10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>1022.5632519841904</v>
       </c>
       <c r="J12" s="5">
         <f>J10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>1053.2401495437164</v>
       </c>
       <c r="K12" s="5">
         <f>K10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>1084.8373540300277</v>
       </c>
       <c r="L12" s="5">
         <f>L10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>1117.3824746509285</v>
       </c>
       <c r="M12" s="5">
         <f>M10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
-        <v/>
+        <v>1150.9039488904566</v>
       </c>
       <c r="N12" s="25">
         <f>SUM(B12:M12)</f>
-        <v/>
+        <v>11799.785578572333</v>
       </c>
     </row>
     <row r="13">
@@ -3582,55 +3582,55 @@
       </c>
       <c r="B13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="C13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="D13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="E13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="F13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="G13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="H13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="I13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="J13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="K13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="L13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="M13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v/>
+        <v>9285.0</v>
       </c>
       <c r="N13" s="25">
         <f>SUM(B13:M13)</f>
-        <v/>
+        <v>111420.0</v>
       </c>
     </row>
     <row r="14">
@@ -3641,55 +3641,55 @@
       </c>
       <c r="B14" s="5">
         <f>B11*'关键假设'!C43</f>
-        <v/>
+        <v>312.0</v>
       </c>
       <c r="C14" s="5">
         <f>C11*'关键假设'!C43</f>
-        <v/>
+        <v>321.36000000000007</v>
       </c>
       <c r="D14" s="5">
         <f>D11*'关键假设'!C43</f>
-        <v/>
+        <v>331.0008000000001</v>
       </c>
       <c r="E14" s="5">
         <f>E11*'关键假设'!C43</f>
-        <v/>
+        <v>340.93082400000003</v>
       </c>
       <c r="F14" s="5">
         <f>F11*'关键假设'!C43</f>
-        <v/>
+        <v>351.15874872</v>
       </c>
       <c r="G14" s="5">
         <f>G11*'关键假设'!C43</f>
-        <v/>
+        <v>361.69351118160006</v>
       </c>
       <c r="H14" s="5">
         <f>H11*'关键假设'!C43</f>
-        <v/>
+        <v>372.54431651704806</v>
       </c>
       <c r="I14" s="5">
         <f>I11*'关键假设'!C43</f>
-        <v/>
+        <v>383.72064601255954</v>
       </c>
       <c r="J14" s="5">
         <f>J11*'关键假设'!C43</f>
-        <v/>
+        <v>395.2322653929363</v>
       </c>
       <c r="K14" s="5">
         <f>K11*'关键假设'!C43</f>
-        <v/>
+        <v>407.0892333547244</v>
       </c>
       <c r="L14" s="5">
         <f>L11*'关键假设'!C43</f>
-        <v/>
+        <v>419.30191035536615</v>
       </c>
       <c r="M14" s="5">
         <f>M11*'关键假设'!C43</f>
-        <v/>
+        <v>431.8809676660272</v>
       </c>
       <c r="N14" s="25">
         <f>SUM(B14:M14)</f>
-        <v/>
+        <v>4427.913223200262</v>
       </c>
     </row>
     <row r="15">
@@ -3700,55 +3700,55 @@
       </c>
       <c r="B15" s="17">
         <f>B11-B12-B13-B14</f>
-        <v/>
+        <v>-28.4375</v>
       </c>
       <c r="C15" s="17">
         <f>C11-C12-C13-C14</f>
-        <v/>
+        <v>249.25937500000197</v>
       </c>
       <c r="D15" s="17">
         <f>D11-D12-D13-D14</f>
-        <v/>
+        <v>535.287156250002</v>
       </c>
       <c r="E15" s="17">
         <f>E11-E12-E13-E14</f>
-        <v/>
+        <v>829.8957709375018</v>
       </c>
       <c r="F15" s="17">
         <f>F11-F12-F13-F14</f>
-        <v/>
+        <v>1133.3426440656272</v>
       </c>
       <c r="G15" s="17">
         <f>G11-G12-G13-G14</f>
-        <v/>
+        <v>1445.8929233875951</v>
       </c>
       <c r="H15" s="17">
         <f>H11-H12-H13-H14</f>
-        <v/>
+        <v>1767.8197110892243</v>
       </c>
       <c r="I15" s="17">
         <f>I11-I12-I13-I14</f>
-        <v/>
+        <v>2099.4043024219013</v>
       </c>
       <c r="J15" s="17">
         <f>J11-J12-J13-J14</f>
-        <v/>
+        <v>2440.9364314945583</v>
       </c>
       <c r="K15" s="17">
         <f>K11-K12-K13-K14</f>
-        <v/>
+        <v>2792.714524439395</v>
       </c>
       <c r="L15" s="17">
         <f>L11-L12-L13-L14</f>
-        <v/>
+        <v>3155.045960172577</v>
       </c>
       <c r="M15" s="17">
         <f>M11-M12-M13-M14</f>
-        <v/>
+        <v>3528.2473389777556</v>
       </c>
       <c r="N15" s="25">
         <f>SUM(B15:M15)</f>
-        <v/>
+        <v>19949.40863823614</v>
       </c>
     </row>
     <row r="16">
@@ -3759,51 +3759,51 @@
       </c>
       <c r="B16" s="5">
         <f>B15</f>
-        <v/>
+        <v>-28.4375</v>
       </c>
       <c r="C16" s="5">
         <f>B16+C15</f>
-        <v/>
+        <v>220.82187500000197</v>
       </c>
       <c r="D16" s="5">
         <f>C16+D15</f>
-        <v/>
+        <v>756.1090312500039</v>
       </c>
       <c r="E16" s="5">
         <f>D16+E15</f>
-        <v/>
+        <v>1586.0048021875057</v>
       </c>
       <c r="F16" s="5">
         <f>E16+F15</f>
-        <v/>
+        <v>2719.347446253133</v>
       </c>
       <c r="G16" s="5">
         <f>F16+G15</f>
-        <v/>
+        <v>4165.240369640728</v>
       </c>
       <c r="H16" s="5">
         <f>G16+H15</f>
-        <v/>
+        <v>5933.0600807299525</v>
       </c>
       <c r="I16" s="5">
         <f>H16+I15</f>
-        <v/>
+        <v>8032.464383151853</v>
       </c>
       <c r="J16" s="5">
         <f>I16+J15</f>
-        <v/>
+        <v>10473.400814646411</v>
       </c>
       <c r="K16" s="5">
         <f>J16+K15</f>
-        <v/>
+        <v>13266.115339085805</v>
       </c>
       <c r="L16" s="5">
         <f>K16+L15</f>
-        <v/>
+        <v>16421.161299258383</v>
       </c>
       <c r="M16" s="5">
         <f>L16+M15</f>
-        <v/>
+        <v>19949.40863823614</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Fix subtotal row text overlapping the amount column
Subtotal rows repeated the full section title (e.g. "Subtotal: 5. Company
& Compliance Setup (mirrors the not-yet-completed Chapter 9 - Legal &
Documentation)"), which overflowed column B far enough to overlap the RM
amount a few columns over in viewers that don't clip overflow the way
Excel does. The full title is already shown in the blue section header
bar directly above each subtotal row, so it was redundant -- shortened
every subtotal/grand-total label to just "Subtotal" / "小计" and "CAPEX
Grand Total" / "OPEX Grand Total", which removes the overflow risk
entirely instead of just patching individual cells.
</commit_message>
<xml_diff>
--- a/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
+++ b/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
@@ -1427,7 +1427,7 @@
     <row r="10">
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>小计：1. 商场租赁 一次性费用 (文件 3.4)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C10" s="16" t="n"/>
@@ -1604,7 +1604,7 @@
     <row r="21">
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>小计：2. 装修工程 (文件 3.8)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C21" s="16" t="n"/>
@@ -1817,7 +1817,7 @@
     <row r="34">
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>小计：3. 店铺设备 (文件 3.9)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C34" s="16" t="n"/>
@@ -1966,7 +1966,7 @@
     <row r="43">
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>小计：4. 支付与系统开办费 (文件 3.10, 5.6)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C43" s="16" t="n"/>
@@ -2119,7 +2119,7 @@
     <row r="52">
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>小计：5. 公司与合规开办费 (呼应待完成的第9章 法律与文件)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C52" s="16" t="n"/>
@@ -2220,7 +2220,7 @@
     <row r="59">
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>小计：6. 首批库存 (文件 3.6 / Decision Log #008，自动按 70/20/10 比例计算)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C59" s="16" t="n"/>
@@ -2289,7 +2289,7 @@
     <row r="64">
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>小计：7. 现金流保护储备 (文件 3.5 现金流保护原则 / Decision Log #018)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C64" s="16" t="n"/>
@@ -2309,7 +2309,7 @@
     <row r="68">
       <c r="B68" s="18" t="inlineStr">
         <is>
-          <t>CAPEX 总计（含现金储备）</t>
+          <t>CAPEX 总计</t>
         </is>
       </c>
       <c r="E68" s="19">
@@ -2474,7 +2474,7 @@
     <row r="11">
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>小计：1. 场地相关 (文件 3.4)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C11" s="17">
@@ -2556,7 +2556,7 @@
     <row r="18">
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>小计：2. 人员成本 (文件 2.16 / 自动引用关键假设)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C18" s="17">
@@ -2606,7 +2606,7 @@
     <row r="23">
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>小计：3. 支付渠道手续费（变动成本，随营收自动计算）</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C23" s="17">
@@ -2674,7 +2674,7 @@
     <row r="30">
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>小计：4. 营销与获客 (文件 2.13, 3.15)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C30" s="17">
@@ -2746,7 +2746,7 @@
     <row r="37">
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>小计：5. 系统与订阅 (文件 4.3-4.4, 3.11)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C37" s="17">
@@ -2822,7 +2822,7 @@
     <row r="44">
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>小计：6. 售后与风险准备 (文件 2.12, 3.13, 3.14 / 呼应第9章法律缺口)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C44" s="17">
@@ -2894,7 +2894,7 @@
     <row r="51">
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>小计：7. 其他行政 (呼应待完成第9章法律与文件)</t>
+          <t>小计</t>
         </is>
       </c>
       <c r="C51" s="17">
@@ -2912,7 +2912,7 @@
     <row r="55">
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>每月固定营运支出总计</t>
+          <t>OPEX 总计</t>
         </is>
       </c>
       <c r="C55" s="19">

</xml_diff>

<commit_message>
Fix sales commission being double-counted in net profit
OPEX Monthly Opex included a flat RM300/month "sales commission (estimate)"
line item in its Staffing Costs subtotal, and that OPEX total flows into
the 12-Month Cash Flow Forecast's net profit formula. The forecast sheet
separately computes a dynamic commission (gross margin x commission rate)
and subtracts that too, so commission was being subtracted twice every
month -- understating net profit by ~RM300/month (RM3,600/year).

The same trap was already correctly avoided for payment processing fees
(that OPEX line is explicitly zeroed with a "kept at 0 to avoid double-
counting" note) but the fix was never applied to the commission line.
Zeroed it out the same way. 12-month net profit moves from RM19,949 to
RM23,549 -- exactly +RM300 x 12, confirming the bug and the fix.
</commit_message>
<xml_diff>
--- a/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
+++ b/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="C6" s="4">
         <f>'CAPEX 开店资本支出'!E68</f>
-        <v>89462.5</v>
+        <v>88712.5</v>
       </c>
     </row>
     <row r="8">
@@ -615,7 +615,7 @@
       </c>
       <c r="C9" s="4">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
     </row>
     <row r="10">
@@ -626,7 +626,7 @@
       </c>
       <c r="C10" s="5">
         <f>'OPEX 每月营运支出'!C56</f>
-        <v>23212.5</v>
+        <v>22462.5</v>
       </c>
     </row>
     <row r="12">
@@ -644,7 +644,7 @@
       </c>
       <c r="C13" s="4">
         <f>'CAPEX 开店资本支出'!E68</f>
-        <v>89462.5</v>
+        <v>88712.5</v>
       </c>
     </row>
     <row r="14">
@@ -684,7 +684,7 @@
       </c>
       <c r="C19" s="5">
         <f>'12个月现金流预测'!N15</f>
-        <v>19949.40863823614</v>
+        <v>23549.408638236142</v>
       </c>
     </row>
     <row r="20">
@@ -695,7 +695,7 @@
       </c>
       <c r="C20" s="5">
         <f>'12个月现金流预测'!M16</f>
-        <v>19949.40863823614</v>
+        <v>23549.40863823614</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
@@ -2296,7 +2296,7 @@
       <c r="D64" s="16" t="n"/>
       <c r="E64" s="17">
         <f>'OPEX 每月营运支出'!C56</f>
-        <v>23212.5</v>
+        <v>22462.5</v>
       </c>
     </row>
     <row r="67">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="E68" s="19">
         <f>E10+E21+E34+E43+E52+E59+E64</f>
-        <v>89462.5</v>
+        <v>88712.5</v>
       </c>
     </row>
     <row r="69">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="E69" s="21">
         <f>'关键假设'!C4-E68</f>
-        <v>-39462.5</v>
+        <v>-38712.5</v>
       </c>
     </row>
     <row r="70">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E70" s="21">
         <f>'关键假设'!C5-E68</f>
-        <v>10537.5</v>
+        <v>11287.5</v>
       </c>
     </row>
   </sheetData>
@@ -2541,15 +2541,15 @@
     <row r="17">
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>销售佣金（估算，实际见现金流预测表按毛利联动）</t>
+          <t>销售佣金（此处保留0，避免与「12个月现金流预测」表按毛利动态计算的佣金重复扣除）</t>
         </is>
       </c>
       <c r="C17" s="22" t="n">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>初期估算值，待首月实际毛利数据校正</t>
+          <t>佣金已在「12个月现金流预测」表按当月毛利×佣金比例自动计算，此处若填数字会被重复扣除两次</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C18" s="17">
         <f>SUM(C15:C17)</f>
-        <v>2560.0</v>
+        <v>2260.0</v>
       </c>
     </row>
     <row r="20">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="C55" s="19">
         <f>C11+C18+C23+C30+C37+C44+C51</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
     </row>
     <row r="56">
@@ -2928,7 +2928,7 @@
       </c>
       <c r="C56" s="21">
         <f>C55*2.5</f>
-        <v>23212.5</v>
+        <v>22462.5</v>
       </c>
     </row>
   </sheetData>
@@ -3582,55 +3582,55 @@
       </c>
       <c r="B13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="C13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="D13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="E13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="F13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="G13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="H13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="I13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="J13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="K13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="L13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="M13" s="5">
         <f>'OPEX 每月营运支出'!C55</f>
-        <v>9285.0</v>
+        <v>8985.0</v>
       </c>
       <c r="N13" s="25">
         <f>SUM(B13:M13)</f>
-        <v>111420.0</v>
+        <v>107820.0</v>
       </c>
     </row>
     <row r="14">
@@ -3700,55 +3700,55 @@
       </c>
       <c r="B15" s="17">
         <f>B11-B12-B13-B14</f>
-        <v>-28.4375</v>
+        <v>271.5625</v>
       </c>
       <c r="C15" s="17">
         <f>C11-C12-C13-C14</f>
-        <v>249.25937500000197</v>
+        <v>549.2593750000019</v>
       </c>
       <c r="D15" s="17">
         <f>D11-D12-D13-D14</f>
-        <v>535.287156250002</v>
+        <v>835.287156250002</v>
       </c>
       <c r="E15" s="17">
         <f>E11-E12-E13-E14</f>
-        <v>829.8957709375018</v>
+        <v>1129.8957709375018</v>
       </c>
       <c r="F15" s="17">
         <f>F11-F12-F13-F14</f>
-        <v>1133.3426440656272</v>
+        <v>1433.3426440656272</v>
       </c>
       <c r="G15" s="17">
         <f>G11-G12-G13-G14</f>
-        <v>1445.8929233875951</v>
+        <v>1745.8929233875951</v>
       </c>
       <c r="H15" s="17">
         <f>H11-H12-H13-H14</f>
-        <v>1767.8197110892243</v>
+        <v>2067.8197110892243</v>
       </c>
       <c r="I15" s="17">
         <f>I11-I12-I13-I14</f>
-        <v>2099.4043024219013</v>
+        <v>2399.4043024219013</v>
       </c>
       <c r="J15" s="17">
         <f>J11-J12-J13-J14</f>
-        <v>2440.9364314945583</v>
+        <v>2740.9364314945583</v>
       </c>
       <c r="K15" s="17">
         <f>K11-K12-K13-K14</f>
-        <v>2792.714524439395</v>
+        <v>3092.714524439395</v>
       </c>
       <c r="L15" s="17">
         <f>L11-L12-L13-L14</f>
-        <v>3155.045960172577</v>
+        <v>3455.045960172577</v>
       </c>
       <c r="M15" s="17">
         <f>M11-M12-M13-M14</f>
-        <v>3528.2473389777556</v>
+        <v>3828.2473389777556</v>
       </c>
       <c r="N15" s="25">
         <f>SUM(B15:M15)</f>
-        <v>19949.40863823614</v>
+        <v>23549.408638236142</v>
       </c>
     </row>
     <row r="16">
@@ -3759,51 +3759,51 @@
       </c>
       <c r="B16" s="5">
         <f>B15</f>
-        <v>-28.4375</v>
+        <v>271.5625</v>
       </c>
       <c r="C16" s="5">
         <f>B16+C15</f>
-        <v>220.82187500000197</v>
+        <v>820.8218750000019</v>
       </c>
       <c r="D16" s="5">
         <f>C16+D15</f>
-        <v>756.1090312500039</v>
+        <v>1656.109031250004</v>
       </c>
       <c r="E16" s="5">
         <f>D16+E15</f>
-        <v>1586.0048021875057</v>
+        <v>2786.0048021875054</v>
       </c>
       <c r="F16" s="5">
         <f>E16+F15</f>
-        <v>2719.347446253133</v>
+        <v>4219.347446253132</v>
       </c>
       <c r="G16" s="5">
         <f>F16+G15</f>
-        <v>4165.240369640728</v>
+        <v>5965.240369640727</v>
       </c>
       <c r="H16" s="5">
         <f>G16+H15</f>
-        <v>5933.0600807299525</v>
+        <v>8033.060080729952</v>
       </c>
       <c r="I16" s="5">
         <f>H16+I15</f>
-        <v>8032.464383151853</v>
+        <v>10432.464383151853</v>
       </c>
       <c r="J16" s="5">
         <f>I16+J15</f>
-        <v>10473.400814646411</v>
+        <v>13173.400814646411</v>
       </c>
       <c r="K16" s="5">
         <f>J16+K15</f>
-        <v>13266.115339085805</v>
+        <v>16266.115339085805</v>
       </c>
       <c r="L16" s="5">
         <f>K16+L15</f>
-        <v>16421.161299258383</v>
+        <v>19721.161299258383</v>
       </c>
       <c r="M16" s="5">
         <f>L16+M15</f>
-        <v>19949.40863823614</v>
+        <v>23549.40863823614</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Add explicit COGS row to forecast and RM6,000/month director fees
- 12-Month Cash Flow Forecast now shows a "Cost of goods sold / stock cost"
  line between Total revenue and Gross margin, so the sheet reads as a clean
  waterfall (Revenue - COGS = Gross margin - fees - OPEX - commission = Net
  profit). COGS = Revenue - Gross margin, computed per month and totalled.

- Added RM6,000/month director fees to OPEX Staffing Costs. This raises
  monthly OPEX to RM14,985 and, because the recommended cash reserve is
  2.5x OPEX, CAPEX total to RM103,712.50. At the current base-case sales
  volume the added draw makes the 12-month net profit -RM48,451, so the
  Summary budget check now flags "exceeds upper bound" -- surfaced for the
  user's decision, not silently absorbed.
</commit_message>
<xml_diff>
--- a/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
+++ b/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="C6" s="4">
         <f>'CAPEX 开店资本支出'!E68</f>
-        <v>88712.5</v>
+        <v>103712.5</v>
       </c>
     </row>
     <row r="8">
@@ -614,8 +614,8 @@
         </is>
       </c>
       <c r="C9" s="4">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
     </row>
     <row r="10">
@@ -625,8 +625,8 @@
         </is>
       </c>
       <c r="C10" s="5">
-        <f>'OPEX 每月营运支出'!C56</f>
-        <v>22462.5</v>
+        <f>'OPEX 每月营运支出'!C57</f>
+        <v>37462.5</v>
       </c>
     </row>
     <row r="12">
@@ -644,7 +644,7 @@
       </c>
       <c r="C13" s="4">
         <f>'CAPEX 开店资本支出'!E68</f>
-        <v>88712.5</v>
+        <v>103712.5</v>
       </c>
     </row>
     <row r="14">
@@ -655,7 +655,7 @@
       </c>
       <c r="C14" t="str">
         <f>IF(C13&lt;='关键假设'!C4,"低于下限，资金充裕",IF(C13&lt;='关键假设'!C5,"落在预算区间内","超出预算上限，需调整假设或增资"))</f>
-        <v>落在预算区间内</v>
+        <v>超出预算上限，需调整假设或增资</v>
       </c>
     </row>
     <row r="17">
@@ -683,8 +683,8 @@
         </is>
       </c>
       <c r="C19" s="5">
-        <f>'12个月现金流预测'!N15</f>
-        <v>23549.408638236142</v>
+        <f>'12个月现金流预测'!N16</f>
+        <v>-48450.59136176386</v>
       </c>
     </row>
     <row r="20">
@@ -694,8 +694,8 @@
         </is>
       </c>
       <c r="C20" s="5">
-        <f>'12个月现金流预测'!M16</f>
-        <v>23549.40863823614</v>
+        <f>'12个月现金流预测'!M17</f>
+        <v>-48450.591361763865</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
@@ -2295,8 +2295,8 @@
       <c r="C64" s="16" t="n"/>
       <c r="D64" s="16" t="n"/>
       <c r="E64" s="17">
-        <f>'OPEX 每月营运支出'!C56</f>
-        <v>22462.5</v>
+        <f>'OPEX 每月营运支出'!C57</f>
+        <v>37462.5</v>
       </c>
     </row>
     <row r="67">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="E68" s="19">
         <f>E10+E21+E34+E43+E52+E59+E64</f>
-        <v>88712.5</v>
+        <v>103712.5</v>
       </c>
     </row>
     <row r="69">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="E69" s="21">
         <f>'关键假设'!C4-E68</f>
-        <v>-38712.5</v>
+        <v>-53712.5</v>
       </c>
     </row>
     <row r="70">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="E70" s="21">
         <f>'关键假设'!C5-E68</f>
-        <v>11287.5</v>
+        <v>-3712.5</v>
       </c>
     </row>
   </sheetData>
@@ -2361,7 +2361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D56"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2509,439 +2509,454 @@
     <row r="15">
       <c r="B15" s="9" t="inlineStr">
         <is>
+          <t>董事袍金/董事酬劳</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>每月从生意中支取的董事酬劳</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
           <t>员工基本工资</t>
         </is>
       </c>
-      <c r="C15" s="14">
+      <c r="C16" s="14">
         <f>'关键假设'!C41</f>
         <v>2000.0</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>引用关键假设表·员工基本工资</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="9" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>EPF/SOCSO/EIS 雇主部分</t>
         </is>
       </c>
-      <c r="C16" s="14">
+      <c r="C17" s="14">
         <f>'关键假设'!C41*'关键假设'!C42</f>
         <v>260.0</v>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>计算式：工资 × 雇主负担比例</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="9" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>销售佣金（此处保留0，避免与「12个月现金流预测」表按毛利动态计算的佣金重复扣除）</t>
         </is>
       </c>
-      <c r="C17" s="22" t="n">
+      <c r="C18" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>佣金已在「12个月现金流预测」表按当月毛利×佣金比例自动计算，此处若填数字会被重复扣除两次</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="15" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>小计</t>
         </is>
       </c>
-      <c r="C18" s="17">
-        <f>SUM(C15:C17)</f>
-        <v>2260.0</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="3" t="inlineStr">
+      <c r="C19" s="17">
+        <f>SUM(C15:C18)</f>
+        <v>8260.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>3. 支付渠道手续费（变动成本，随营收自动计算）</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="13" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C22" s="13" t="inlineStr">
         <is>
           <t>每月金额 (RM)</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="9" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>说明：手续费为变动成本，已在「12个月现金流预测」按渠道占比与费率自动计算，此处填0避免重复计算</t>
         </is>
       </c>
-      <c r="C22" s="22" t="n">
+      <c r="C23" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>如需查看月度手续费金额，见「12个月现金流预测」表</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="15" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t>小计</t>
         </is>
       </c>
-      <c r="C23" s="17">
-        <f>SUM(C22:C22)</f>
+      <c r="C24" s="17">
+        <f>SUM(C23:C23)</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="3" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>4. 营销与获客 (文件 2.13, 3.15)</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="13" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
+      <c r="C27" s="13" t="inlineStr">
         <is>
           <t>每月金额 (RM)</t>
         </is>
       </c>
-      <c r="D26" s="13" t="inlineStr">
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Facebook 广告</t>
-        </is>
-      </c>
-      <c r="C27" s="22" t="n">
-        <v>500</v>
-      </c>
-      <c r="D27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>TikTok 内容/广告</t>
+          <t>Facebook 广告</t>
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="D28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="B29" s="9" t="inlineStr">
         <is>
+          <t>TikTok 内容/广告</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="n">
+        <v>300</v>
+      </c>
+      <c r="D29" s="7" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="9" t="inlineStr">
+        <is>
           <t>开业/促销物料（首3个月后转为常态小额预算）</t>
         </is>
       </c>
-      <c r="C29" s="22" t="n">
+      <c r="C30" s="22" t="n">
         <v>200</v>
       </c>
-      <c r="D29" s="7" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="15" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="15" t="inlineStr">
         <is>
           <t>小计</t>
         </is>
       </c>
-      <c r="C30" s="17">
-        <f>SUM(C27:C29)</f>
+      <c r="C31" s="17">
+        <f>SUM(C28:C30)</f>
         <v>1000.0</v>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" s="3" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>5. 系统与订阅 (文件 4.3-4.4, 3.11)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" s="13" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C33" s="13" t="inlineStr">
+      <c r="C34" s="13" t="inlineStr">
         <is>
           <t>每月金额 (RM)</t>
         </is>
       </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>Google Sheets（官方库存/记录方案，免费-约RM300/年按月折算）</t>
-        </is>
-      </c>
-      <c r="C34" s="22" t="n">
-        <v>25</v>
-      </c>
-      <c r="D34" s="7" t="inlineStr">
-        <is>
-          <t>文件4.4：Decision Log #007已定为免费/低成本方案</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>网站维护/域名/主机</t>
+          <t>Google Sheets（官方库存/记录方案，免费-约RM300/年按月折算）</t>
         </is>
       </c>
       <c r="C35" s="22" t="n">
-        <v>100</v>
-      </c>
-      <c r="D35" s="7" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>文件4.4：Decision Log #007已定为免费/低成本方案</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="B36" s="9" t="inlineStr">
         <is>
+          <t>网站维护/域名/主机</t>
+        </is>
+      </c>
+      <c r="C36" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D36" s="7" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="9" t="inlineStr">
+        <is>
           <t>WhatsApp Business（免费，如用第三方工具另计）</t>
         </is>
       </c>
-      <c r="C36" s="22" t="n">
+      <c r="C37" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D36" s="7" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="15" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>小计</t>
         </is>
       </c>
-      <c r="C37" s="17">
-        <f>SUM(C34:C36)</f>
+      <c r="C38" s="17">
+        <f>SUM(C35:C37)</f>
         <v>125.0</v>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" s="3" t="inlineStr">
+    <row r="40">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>6. 售后与风险准备 (文件 2.12, 3.13, 3.14 / 呼应第9章法律缺口)</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" s="13" t="inlineStr">
+    <row r="41">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C40" s="13" t="inlineStr">
+      <c r="C41" s="13" t="inlineStr">
         <is>
           <t>每月金额 (RM)</t>
         </is>
       </c>
-      <c r="D40" s="13" t="inlineStr">
+      <c r="D41" s="13" t="inlineStr">
         <is>
           <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>维修/售后处理准备金</t>
-        </is>
-      </c>
-      <c r="C41" s="22" t="n">
-        <v>300</v>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>对应外部维修商合作费用及非原厂保修处理</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="9" t="inlineStr">
         <is>
-          <t>保险分摊（如决定购买，见文件3.14）</t>
+          <t>维修/售后处理准备金</t>
         </is>
       </c>
       <c r="C42" s="22" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>暂不购买，先研究；决定后按年保费/12填入</t>
+          <t>对应外部维修商合作费用及非原厂保修处理</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="9" t="inlineStr">
         <is>
+          <t>保险分摊（如决定购买，见文件3.14）</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>暂不购买，先研究；决定后按年保费/12填入</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
           <t>坏账/退换损耗准备（约营收0.5%，估算值）</t>
         </is>
       </c>
-      <c r="C43" s="22" t="n">
+      <c r="C44" s="22" t="n">
         <v>150</v>
       </c>
-      <c r="D43" s="7" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="B44" s="15" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>小计</t>
         </is>
       </c>
-      <c r="C44" s="17">
-        <f>SUM(C41:C43)</f>
+      <c r="C45" s="17">
+        <f>SUM(C42:C44)</f>
         <v>450.0</v>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" s="3" t="inlineStr">
+    <row r="47">
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>7. 其他行政 (呼应待完成第9章法律与文件)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" s="13" t="inlineStr">
+    <row r="48">
+      <c r="B48" s="13" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="C47" s="13" t="inlineStr">
+      <c r="C48" s="13" t="inlineStr">
         <is>
           <t>每月金额 (RM)</t>
         </is>
       </c>
-      <c r="D47" s="13" t="inlineStr">
+      <c r="D48" s="13" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>会计/记账服务</t>
-        </is>
-      </c>
-      <c r="C48" s="22" t="n">
-        <v>250</v>
-      </c>
-      <c r="D48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>银行手续费/其他行政杂费</t>
+          <t>会计/记账服务</t>
         </is>
       </c>
       <c r="C49" s="22" t="n">
-        <v>50</v>
+        <v>250</v>
       </c>
       <c r="D49" s="7" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="B50" s="9" t="inlineStr">
         <is>
+          <t>银行手续费/其他行政杂费</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="D50" s="7" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="B51" s="9" t="inlineStr">
+        <is>
           <t>LHDN e-Invoice / SST 合规预留（未达门槛前可填0）</t>
         </is>
       </c>
-      <c r="C50" s="22" t="n">
+      <c r="C51" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D50" s="7" t="inlineStr">
+      <c r="D51" s="7" t="inlineStr">
         <is>
           <t>营业额达SST门槛(RM500k)或e-Invoice强制阶段前预留</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="B51" s="15" t="inlineStr">
+    <row r="52">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>小计</t>
         </is>
       </c>
-      <c r="C51" s="17">
-        <f>SUM(C48:C50)</f>
+      <c r="C52" s="17">
+        <f>SUM(C49:C51)</f>
         <v>300.0</v>
       </c>
     </row>
-    <row r="54">
-      <c r="B54" s="3" t="inlineStr">
+    <row r="55">
+      <c r="B55" s="3" t="inlineStr">
         <is>
           <t>OPEX 总计</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="B55" s="18" t="inlineStr">
+    <row r="56">
+      <c r="B56" s="18" t="inlineStr">
         <is>
           <t>OPEX 总计</t>
         </is>
       </c>
-      <c r="C55" s="19">
-        <f>C11+C18+C23+C30+C37+C44+C51</f>
-        <v>8985.0</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" s="20" t="inlineStr">
+      <c r="C56" s="19">
+        <f>C11+C19+C24+C31+C38+C45+C52</f>
+        <v>14985.0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="20" t="inlineStr">
         <is>
           <t>建议现金储备（2.5个月固定成本，文件3.5要求2-3个月）</t>
         </is>
       </c>
-      <c r="C56" s="21">
-        <f>C55*2.5</f>
-        <v>22462.5</v>
+      <c r="C57" s="21">
+        <f>C56*2.5</f>
+        <v>37462.5</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B33:D33"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B46:D46"/>
-    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B26:D26"/>
+    <mergeCell ref="B40:D40"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B47:D47"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2953,7 +2968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3459,355 +3474,414 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>销货成本/进货成本 (RM) = 营收 − 毛利</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>B10-B12</f>
+        <v>52350.0</v>
+      </c>
+      <c r="C11" s="5">
+        <f>C10-C12</f>
+        <v>53920.50000000001</v>
+      </c>
+      <c r="D11" s="5">
+        <f>D10-D12</f>
+        <v>55538.115000000005</v>
+      </c>
+      <c r="E11" s="5">
+        <f>E10-E12</f>
+        <v>57204.25845</v>
+      </c>
+      <c r="F11" s="5">
+        <f>F10-F12</f>
+        <v>58920.386203500006</v>
+      </c>
+      <c r="G11" s="5">
+        <f>G10-G12</f>
+        <v>60687.99778960501</v>
+      </c>
+      <c r="H11" s="5">
+        <f>H10-H12</f>
+        <v>62508.637723293155</v>
+      </c>
+      <c r="I11" s="5">
+        <f>I10-I12</f>
+        <v>64383.89685499195</v>
+      </c>
+      <c r="J11" s="5">
+        <f>J10-J12</f>
+        <v>66315.41376064174</v>
+      </c>
+      <c r="K11" s="5">
+        <f>K10-K12</f>
+        <v>68304.87617346096</v>
+      </c>
+      <c r="L11" s="5">
+        <f>L10-L12</f>
+        <v>70354.0224586648</v>
+      </c>
+      <c r="M11" s="5">
+        <f>M10-M12</f>
+        <v>72464.64313242475</v>
+      </c>
+      <c r="N11" s="25">
+        <f>SUM(B11:M11)</f>
+        <v>742952.7475465825</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>估算毛利 (RM)  新机/二手机/配件加权</t>
         </is>
       </c>
-      <c r="B11" s="5">
+      <c r="B12" s="5">
         <f>(B6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(B9*'关键假设'!C15)</f>
         <v>10400.0</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C12" s="5">
         <f>(C6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(C9*'关键假设'!C15)</f>
         <v>10712.000000000002</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D12" s="5">
         <f>(D6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(D9*'关键假设'!C15)</f>
         <v>11033.360000000002</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E12" s="5">
         <f>(E6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(E9*'关键假设'!C15)</f>
         <v>11364.360800000002</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F12" s="5">
         <f>(F6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(F9*'关键假设'!C15)</f>
         <v>11705.291624000001</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G12" s="5">
         <f>(G6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(G9*'关键假设'!C15)</f>
         <v>12056.450372720003</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H12" s="5">
         <f>(H6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(H9*'关键假设'!C15)</f>
         <v>12418.143883901603</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I12" s="5">
         <f>(I6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(I9*'关键假设'!C15)</f>
         <v>12790.688200418652</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J12" s="5">
         <f>(J6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(J9*'关键假设'!C15)</f>
         <v>13174.408846431212</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K12" s="5">
         <f>(K6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(K9*'关键假设'!C15)</f>
         <v>13569.641111824147</v>
       </c>
-      <c r="L11" s="5">
+      <c r="L12" s="5">
         <f>(L6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(L9*'关键假设'!C15)</f>
         <v>13976.730345178872</v>
       </c>
-      <c r="M11" s="5">
+      <c r="M12" s="5">
         <f>(M6*(('关键假设'!C8/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C13+('关键假设'!C9/('关键假设'!C8+'关键假设'!C9))*'关键假设'!C14))+(M9*'关键假设'!C15)</f>
         <v>14396.032255534239</v>
       </c>
-      <c r="N11" s="25">
-        <f>SUM(B11:M11)</f>
+      <c r="N12" s="25">
+        <f>SUM(B12:M12)</f>
         <v>147597.10744000872</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>支付手续费 (RM)</t>
         </is>
       </c>
-      <c r="B12" s="5">
+      <c r="B13" s="5">
         <f>B10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>831.4375</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C13" s="5">
         <f>C10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>856.3806250000001</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D13" s="5">
         <f>D10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>882.07204375</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E13" s="5">
         <f>E10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>908.5342050625001</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F13" s="5">
         <f>F10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>935.7902312143751</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G13" s="5">
         <f>G10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>963.8639381508065</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H13" s="5">
         <f>H10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>992.7798562953305</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I13" s="5">
         <f>I10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>1022.5632519841904</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J13" s="5">
         <f>J10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>1053.2401495437164</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K13" s="5">
         <f>K10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>1084.8373540300277</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L13" s="5">
         <f>L10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>1117.3824746509285</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M13" s="5">
         <f>M10*('关键假设'!C32*'关键假设'!C35+'关键假设'!C33*'关键假设'!C36+'关键假设'!C34*'关键假设'!C37)</f>
         <v>1150.9039488904566</v>
       </c>
-      <c r="N12" s="25">
-        <f>SUM(B12:M12)</f>
-        <v>11799.785578572333</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>每月固定营运支出 OPEX (RM)</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="C13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="D13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="E13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="F13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="G13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="H13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="I13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="J13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="K13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="L13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
-      <c r="M13" s="5">
-        <f>'OPEX 每月营运支出'!C55</f>
-        <v>8985.0</v>
-      </c>
       <c r="N13" s="25">
         <f>SUM(B13:M13)</f>
-        <v>107820.0</v>
+        <v>11799.785578572333</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>销售佣金 (毛利的比例)</t>
+          <t>每月固定营运支出 OPEX (RM)</t>
         </is>
       </c>
       <c r="B14" s="5">
-        <f>B11*'关键假设'!C43</f>
-        <v>312.0</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="C14" s="5">
-        <f>C11*'关键假设'!C43</f>
-        <v>321.36000000000007</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="D14" s="5">
-        <f>D11*'关键假设'!C43</f>
-        <v>331.0008000000001</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="E14" s="5">
-        <f>E11*'关键假设'!C43</f>
-        <v>340.93082400000003</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="F14" s="5">
-        <f>F11*'关键假设'!C43</f>
-        <v>351.15874872</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="G14" s="5">
-        <f>G11*'关键假设'!C43</f>
-        <v>361.69351118160006</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="H14" s="5">
-        <f>H11*'关键假设'!C43</f>
-        <v>372.54431651704806</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="I14" s="5">
-        <f>I11*'关键假设'!C43</f>
-        <v>383.72064601255954</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="J14" s="5">
-        <f>J11*'关键假设'!C43</f>
-        <v>395.2322653929363</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="K14" s="5">
-        <f>K11*'关键假设'!C43</f>
-        <v>407.0892333547244</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="L14" s="5">
-        <f>L11*'关键假设'!C43</f>
-        <v>419.30191035536615</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="M14" s="5">
-        <f>M11*'关键假设'!C43</f>
-        <v>431.8809676660272</v>
+        <f>'OPEX 每月营运支出'!C56</f>
+        <v>14985.0</v>
       </c>
       <c r="N14" s="25">
         <f>SUM(B14:M14)</f>
-        <v>4427.913223200262</v>
+        <v>179820.0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
-        <is>
-          <t>净利润 (RM) = 毛利 − 手续费 − OPEX − 佣金</t>
-        </is>
-      </c>
-      <c r="B15" s="17">
-        <f>B11-B12-B13-B14</f>
-        <v>271.5625</v>
-      </c>
-      <c r="C15" s="17">
-        <f>C11-C12-C13-C14</f>
-        <v>549.2593750000019</v>
-      </c>
-      <c r="D15" s="17">
-        <f>D11-D12-D13-D14</f>
-        <v>835.287156250002</v>
-      </c>
-      <c r="E15" s="17">
-        <f>E11-E12-E13-E14</f>
-        <v>1129.8957709375018</v>
-      </c>
-      <c r="F15" s="17">
-        <f>F11-F12-F13-F14</f>
-        <v>1433.3426440656272</v>
-      </c>
-      <c r="G15" s="17">
-        <f>G11-G12-G13-G14</f>
-        <v>1745.8929233875951</v>
-      </c>
-      <c r="H15" s="17">
-        <f>H11-H12-H13-H14</f>
-        <v>2067.8197110892243</v>
-      </c>
-      <c r="I15" s="17">
-        <f>I11-I12-I13-I14</f>
-        <v>2399.4043024219013</v>
-      </c>
-      <c r="J15" s="17">
-        <f>J11-J12-J13-J14</f>
-        <v>2740.9364314945583</v>
-      </c>
-      <c r="K15" s="17">
-        <f>K11-K12-K13-K14</f>
-        <v>3092.714524439395</v>
-      </c>
-      <c r="L15" s="17">
-        <f>L11-L12-L13-L14</f>
-        <v>3455.045960172577</v>
-      </c>
-      <c r="M15" s="17">
-        <f>M11-M12-M13-M14</f>
-        <v>3828.2473389777556</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>销售佣金 (毛利的比例)</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>B12*'关键假设'!C43</f>
+        <v>312.0</v>
+      </c>
+      <c r="C15" s="5">
+        <f>C12*'关键假设'!C43</f>
+        <v>321.36000000000007</v>
+      </c>
+      <c r="D15" s="5">
+        <f>D12*'关键假设'!C43</f>
+        <v>331.0008000000001</v>
+      </c>
+      <c r="E15" s="5">
+        <f>E12*'关键假设'!C43</f>
+        <v>340.93082400000003</v>
+      </c>
+      <c r="F15" s="5">
+        <f>F12*'关键假设'!C43</f>
+        <v>351.15874872</v>
+      </c>
+      <c r="G15" s="5">
+        <f>G12*'关键假设'!C43</f>
+        <v>361.69351118160006</v>
+      </c>
+      <c r="H15" s="5">
+        <f>H12*'关键假设'!C43</f>
+        <v>372.54431651704806</v>
+      </c>
+      <c r="I15" s="5">
+        <f>I12*'关键假设'!C43</f>
+        <v>383.72064601255954</v>
+      </c>
+      <c r="J15" s="5">
+        <f>J12*'关键假设'!C43</f>
+        <v>395.2322653929363</v>
+      </c>
+      <c r="K15" s="5">
+        <f>K12*'关键假设'!C43</f>
+        <v>407.0892333547244</v>
+      </c>
+      <c r="L15" s="5">
+        <f>L12*'关键假设'!C43</f>
+        <v>419.30191035536615</v>
+      </c>
+      <c r="M15" s="5">
+        <f>M12*'关键假设'!C43</f>
+        <v>431.8809676660272</v>
       </c>
       <c r="N15" s="25">
         <f>SUM(B15:M15)</f>
-        <v>23549.408638236142</v>
+        <v>4427.913223200262</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>净利润 (RM) = 毛利 − 手续费 − OPEX − 佣金</t>
+        </is>
+      </c>
+      <c r="B16" s="17">
+        <f>B12-B13-B14-B15</f>
+        <v>-5728.4375</v>
+      </c>
+      <c r="C16" s="17">
+        <f>C12-C13-C14-C15</f>
+        <v>-5450.740624999998</v>
+      </c>
+      <c r="D16" s="17">
+        <f>D12-D13-D14-D15</f>
+        <v>-5164.712843749998</v>
+      </c>
+      <c r="E16" s="17">
+        <f>E12-E13-E14-E15</f>
+        <v>-4870.104229062498</v>
+      </c>
+      <c r="F16" s="17">
+        <f>F12-F13-F14-F15</f>
+        <v>-4566.657355934373</v>
+      </c>
+      <c r="G16" s="17">
+        <f>G12-G13-G14-G15</f>
+        <v>-4254.107076612405</v>
+      </c>
+      <c r="H16" s="17">
+        <f>H12-H13-H14-H15</f>
+        <v>-3932.1802889107757</v>
+      </c>
+      <c r="I16" s="17">
+        <f>I12-I13-I14-I15</f>
+        <v>-3600.5956975780987</v>
+      </c>
+      <c r="J16" s="17">
+        <f>J12-J13-J14-J15</f>
+        <v>-3259.0635685054417</v>
+      </c>
+      <c r="K16" s="17">
+        <f>K12-K13-K14-K15</f>
+        <v>-2907.285475560605</v>
+      </c>
+      <c r="L16" s="17">
+        <f>L12-L13-L14-L15</f>
+        <v>-2544.954039827423</v>
+      </c>
+      <c r="M16" s="17">
+        <f>M12-M13-M14-M15</f>
+        <v>-2171.7526610222444</v>
+      </c>
+      <c r="N16" s="25">
+        <f>SUM(B16:M16)</f>
+        <v>-48450.59136176386</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>累计净现金流 (RM，起点为0，未计CAPEX)</t>
         </is>
       </c>
-      <c r="B16" s="5">
-        <f>B15</f>
-        <v>271.5625</v>
-      </c>
-      <c r="C16" s="5">
-        <f>B16+C15</f>
-        <v>820.8218750000019</v>
-      </c>
-      <c r="D16" s="5">
-        <f>C16+D15</f>
-        <v>1656.109031250004</v>
-      </c>
-      <c r="E16" s="5">
-        <f>D16+E15</f>
-        <v>2786.0048021875054</v>
-      </c>
-      <c r="F16" s="5">
-        <f>E16+F15</f>
-        <v>4219.347446253132</v>
-      </c>
-      <c r="G16" s="5">
-        <f>F16+G15</f>
-        <v>5965.240369640727</v>
-      </c>
-      <c r="H16" s="5">
-        <f>G16+H15</f>
-        <v>8033.060080729952</v>
-      </c>
-      <c r="I16" s="5">
-        <f>H16+I15</f>
-        <v>10432.464383151853</v>
-      </c>
-      <c r="J16" s="5">
-        <f>I16+J15</f>
-        <v>13173.400814646411</v>
-      </c>
-      <c r="K16" s="5">
-        <f>J16+K15</f>
-        <v>16266.115339085805</v>
-      </c>
-      <c r="L16" s="5">
-        <f>K16+L15</f>
-        <v>19721.161299258383</v>
-      </c>
-      <c r="M16" s="5">
-        <f>L16+M15</f>
-        <v>23549.40863823614</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="B17" s="5">
+        <f>B16</f>
+        <v>-5728.4375</v>
+      </c>
+      <c r="C17" s="5">
+        <f>B17+C16</f>
+        <v>-11179.178124999999</v>
+      </c>
+      <c r="D17" s="5">
+        <f>C17+D16</f>
+        <v>-16343.890968749996</v>
+      </c>
+      <c r="E17" s="5">
+        <f>D17+E16</f>
+        <v>-21213.995197812495</v>
+      </c>
+      <c r="F17" s="5">
+        <f>E17+F16</f>
+        <v>-25780.65255374687</v>
+      </c>
+      <c r="G17" s="5">
+        <f>F17+G16</f>
+        <v>-30034.759630359273</v>
+      </c>
+      <c r="H17" s="5">
+        <f>G17+H16</f>
+        <v>-33966.93991927005</v>
+      </c>
+      <c r="I17" s="5">
+        <f>H17+I16</f>
+        <v>-37567.53561684815</v>
+      </c>
+      <c r="J17" s="5">
+        <f>I17+J16</f>
+        <v>-40826.599185353596</v>
+      </c>
+      <c r="K17" s="5">
+        <f>J17+K16</f>
+        <v>-43733.8846609142</v>
+      </c>
+      <c r="L17" s="5">
+        <f>K17+L16</f>
+        <v>-46278.838700741624</v>
+      </c>
+      <c r="M17" s="5">
+        <f>L17+M16</f>
+        <v>-48450.591361763865</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Decision Log #024 验证标准：连续3个月净利润&gt;0 且累计净现金流为正</t>
         </is>
@@ -3815,10 +3889,10 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A18:N18"/>
+    <mergeCell ref="A19:N19"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <conditionalFormatting sqref="B15:M15">
+  <conditionalFormatting sqref="B16:M16">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -3826,7 +3900,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B16:N16">
+  <conditionalFormatting sqref="B17:N17">
     <cfRule type="cellIs" priority="3" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
Make director fees an editable Key Assumptions cell
Moved the RM6,000/month director fee from a hardcoded OPEX line into a
yellow editable cell in Key Assumptions ("Director fees (monthly)"); the
OPEX Staffing Costs line now references it by formula. Editing the single
assumption cell recalculates OPEX, the 2.5x cash reserve, CAPEX total,
12-month net profit and the budget verdict. Verified across RM0-6,000: the
whole chain tracks correctly and the budget check flips from "exceeds upper
bound" (RM6k) to "within range" (<=RM4k).
</commit_message>
<xml_diff>
--- a/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
+++ b/sun-smart/finance/SUN_SMART_CAPEX_OPEX.xlsx
@@ -836,7 +836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1254,6 +1254,21 @@
       <c r="D43" s="7" t="inlineStr">
         <is>
           <t>假设值，需与员工另行约定</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="9" t="inlineStr">
+        <is>
+          <t>董事袍金（每月）</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>每月董事酬劳。在此处修改可测试不同金额；建议初期取较低值，待每月毛利稳定超过固定成本后再调高</t>
         </is>
       </c>
     </row>
@@ -2512,12 +2527,13 @@
           <t>董事袍金/董事酬劳</t>
         </is>
       </c>
-      <c r="C15" s="22" t="n">
-        <v>6000</v>
+      <c r="C15" s="14">
+        <f>'关键假设'!C44</f>
+        <v>6000.0</v>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>每月从生意中支取的董事酬劳</t>
+          <t>引用关键假设表·董事袍金，在那里修改金额即可</t>
         </is>
       </c>
     </row>

</xml_diff>